<commit_message>
Issue of warnings popping up fixed
</commit_message>
<xml_diff>
--- a/docs/TestPlan.xlsx
+++ b/docs/TestPlan.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="153">
   <si>
     <t>Test Planner and Tracker</t>
   </si>
@@ -71,9 +71,6 @@
   </si>
   <si>
     <t>Successful authentication and redirection to user dashboard</t>
-  </si>
-  <si>
-    <t>Whenever we reach the entry point of the frontend, two errors always pops up at the bottom that says user not authenticated as well as authentication required</t>
   </si>
   <si>
     <t>Implies not part of this Release</t>
@@ -817,7 +814,7 @@
     <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
@@ -833,7 +830,7 @@
     <xf borderId="3" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -1267,12 +1264,10 @@
       <c r="F3" s="14"/>
       <c r="G3" s="15"/>
       <c r="H3" s="16"/>
-      <c r="I3" s="13" t="s">
-        <v>17</v>
-      </c>
+      <c r="I3" s="13"/>
       <c r="K3" s="17"/>
       <c r="L3" s="18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1">
@@ -1284,13 +1279,13 @@
         <v>13</v>
       </c>
       <c r="C4" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="E4" s="13" t="s">
         <v>20</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>21</v>
       </c>
       <c r="F4" s="21"/>
       <c r="G4" s="21"/>
@@ -1298,7 +1293,7 @@
       <c r="I4" s="21"/>
       <c r="K4" s="22"/>
       <c r="L4" s="18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" ht="12.75" customHeight="1">
@@ -1310,13 +1305,13 @@
         <v>13</v>
       </c>
       <c r="C5" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="E5" s="20" t="s">
         <v>24</v>
-      </c>
-      <c r="E5" s="20" t="s">
-        <v>25</v>
       </c>
       <c r="F5" s="21"/>
       <c r="G5" s="21"/>
@@ -1324,7 +1319,7 @@
       <c r="I5" s="21"/>
       <c r="K5" s="23"/>
       <c r="L5" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1">
@@ -1333,16 +1328,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="D6" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="E6" s="20" t="s">
         <v>29</v>
-      </c>
-      <c r="E6" s="20" t="s">
-        <v>30</v>
       </c>
       <c r="F6" s="21"/>
       <c r="G6" s="21"/>
@@ -1355,16 +1350,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="20" t="s">
-        <v>28</v>
-      </c>
       <c r="D7" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="20" t="s">
         <v>31</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>32</v>
       </c>
       <c r="F7" s="21"/>
       <c r="G7" s="21"/>
@@ -1377,16 +1372,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C8" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="E8" s="20" t="s">
         <v>34</v>
-      </c>
-      <c r="E8" s="20" t="s">
-        <v>35</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="21"/>
@@ -1399,16 +1394,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="20" t="s">
+      <c r="E9" s="20" t="s">
         <v>37</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>38</v>
       </c>
       <c r="F9" s="21"/>
       <c r="G9" s="21"/>
@@ -1421,16 +1416,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D10" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="20" t="s">
         <v>39</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>40</v>
       </c>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
@@ -1443,16 +1438,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="D11" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="E11" s="20" t="s">
         <v>43</v>
-      </c>
-      <c r="E11" s="20" t="s">
-        <v>44</v>
       </c>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
@@ -1465,16 +1460,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="E12" s="20" t="s">
         <v>46</v>
-      </c>
-      <c r="E12" s="20" t="s">
-        <v>47</v>
       </c>
       <c r="F12" s="21"/>
       <c r="G12" s="21"/>
@@ -1484,16 +1479,16 @@
     <row r="13" ht="12.75" customHeight="1">
       <c r="A13" s="19"/>
       <c r="B13" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D13" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="20" t="s">
         <v>48</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>49</v>
       </c>
       <c r="F13" s="21"/>
       <c r="G13" s="21"/>
@@ -1506,16 +1501,16 @@
         <v>11</v>
       </c>
       <c r="B14" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="D14" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="E14" s="20" t="s">
         <v>52</v>
-      </c>
-      <c r="E14" s="20" t="s">
-        <v>53</v>
       </c>
       <c r="F14" s="21"/>
       <c r="G14" s="21"/>
@@ -1528,16 +1523,16 @@
         <v>12</v>
       </c>
       <c r="B15" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="D15" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="E15" s="20" t="s">
         <v>56</v>
-      </c>
-      <c r="E15" s="20" t="s">
-        <v>57</v>
       </c>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
@@ -1550,16 +1545,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C16" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="20" t="s">
         <v>58</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="E16" s="20" t="s">
-        <v>59</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="21"/>
@@ -1572,16 +1567,16 @@
         <v>14</v>
       </c>
       <c r="B17" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="20" t="s">
+      <c r="E17" s="20" t="s">
         <v>61</v>
-      </c>
-      <c r="E17" s="20" t="s">
-        <v>62</v>
       </c>
       <c r="F17" s="21"/>
       <c r="G17" s="21"/>
@@ -1594,16 +1589,16 @@
         <v>15</v>
       </c>
       <c r="B18" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="D18" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="E18" s="20" t="s">
         <v>65</v>
-      </c>
-      <c r="E18" s="20" t="s">
-        <v>66</v>
       </c>
       <c r="F18" s="21"/>
       <c r="G18" s="21"/>
@@ -1616,16 +1611,16 @@
         <v>16</v>
       </c>
       <c r="B19" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="D19" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="E19" s="20" t="s">
         <v>69</v>
-      </c>
-      <c r="E19" s="20" t="s">
-        <v>70</v>
       </c>
       <c r="F19" s="21"/>
       <c r="G19" s="21"/>
@@ -1638,16 +1633,16 @@
         <v>17</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C20" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" s="20" t="s">
         <v>71</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="E20" s="20" t="s">
-        <v>72</v>
       </c>
       <c r="F20" s="21"/>
       <c r="G20" s="21"/>
@@ -1660,16 +1655,16 @@
         <v>18</v>
       </c>
       <c r="B21" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="D21" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="E21" s="20" t="s">
         <v>75</v>
-      </c>
-      <c r="E21" s="20" t="s">
-        <v>76</v>
       </c>
       <c r="F21" s="21"/>
       <c r="G21" s="21"/>
@@ -1682,16 +1677,16 @@
         <v>19</v>
       </c>
       <c r="B22" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="D22" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="D22" s="20" t="s">
+      <c r="E22" s="20" t="s">
         <v>79</v>
-      </c>
-      <c r="E22" s="20" t="s">
-        <v>80</v>
       </c>
       <c r="F22" s="21"/>
       <c r="G22" s="21"/>
@@ -1704,16 +1699,16 @@
         <v>20</v>
       </c>
       <c r="B23" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" s="20" t="s">
+      <c r="E23" s="20" t="s">
         <v>82</v>
-      </c>
-      <c r="E23" s="20" t="s">
-        <v>83</v>
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
@@ -1726,16 +1721,16 @@
         <v>21</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D24" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="20" t="s">
         <v>84</v>
-      </c>
-      <c r="E24" s="20" t="s">
-        <v>85</v>
       </c>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
@@ -1748,16 +1743,16 @@
         <v>22</v>
       </c>
       <c r="B25" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="20" t="s">
+      <c r="E25" s="20" t="s">
         <v>87</v>
-      </c>
-      <c r="E25" s="20" t="s">
-        <v>88</v>
       </c>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
@@ -1770,16 +1765,16 @@
         <v>23</v>
       </c>
       <c r="B26" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="D26" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="D26" s="20" t="s">
+      <c r="E26" s="20" t="s">
         <v>91</v>
-      </c>
-      <c r="E26" s="20" t="s">
-        <v>92</v>
       </c>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
@@ -1792,16 +1787,16 @@
         <v>24</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D27" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="E27" s="20" t="s">
         <v>93</v>
-      </c>
-      <c r="E27" s="20" t="s">
-        <v>94</v>
       </c>
       <c r="F27" s="21"/>
       <c r="G27" s="21"/>
@@ -1814,16 +1809,16 @@
         <v>25</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D28" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="20" t="s">
         <v>95</v>
-      </c>
-      <c r="E28" s="20" t="s">
-        <v>96</v>
       </c>
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
@@ -1925,7 +1920,7 @@
       <c r="B38" s="26"/>
       <c r="C38" s="26"/>
       <c r="K38" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Q38" s="4"/>
       <c r="R38" s="4"/>
@@ -1937,7 +1932,7 @@
       <c r="B39" s="26"/>
       <c r="C39" s="26"/>
       <c r="K39" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
@@ -1949,7 +1944,7 @@
       <c r="B40" s="26"/>
       <c r="C40" s="26"/>
       <c r="K40" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="Q40" s="4"/>
       <c r="R40" s="4"/>
@@ -1961,7 +1956,7 @@
       <c r="B41" s="26"/>
       <c r="C41" s="26"/>
       <c r="K41" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q41" s="4"/>
       <c r="R41" s="4"/>
@@ -1973,7 +1968,7 @@
       <c r="B42" s="26"/>
       <c r="C42" s="26"/>
       <c r="K42" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q42" s="4"/>
       <c r="R42" s="4"/>
@@ -1985,7 +1980,7 @@
       <c r="B43" s="26"/>
       <c r="C43" s="26"/>
       <c r="K43" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q43" s="4"/>
       <c r="R43" s="4"/>
@@ -6889,83 +6884,83 @@
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
       <c r="B1" s="27" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" ht="12.75" customHeight="1"/>
     <row r="3" ht="12.75" customHeight="1">
       <c r="B3" s="28" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="B4" s="28" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="B5" s="28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="B6" s="28" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="B7" s="28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="B8" s="28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" ht="12.75" customHeight="1">
       <c r="B9" s="28" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" ht="12.75" customHeight="1">
       <c r="B10" s="28" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="B11" s="28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" ht="12.75" customHeight="1">
       <c r="B12" s="28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" ht="12.75" customHeight="1">
       <c r="B13" s="28" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1">
       <c r="B14" s="28" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" ht="12.75" customHeight="1">
       <c r="B15" s="28" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" ht="12.75" customHeight="1">
       <c r="B16" s="28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" ht="12.75" customHeight="1">
       <c r="B17" s="28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" ht="12.75" customHeight="1"/>
@@ -7979,7 +7974,7 @@
     <row r="1" ht="12.75" customHeight="1"/>
     <row r="2" ht="12.75" customHeight="1">
       <c r="A2" s="29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
@@ -7987,20 +7982,20 @@
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="26"/>
       <c r="B3" s="30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C3" s="26"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="26"/>
       <c r="B4" s="31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C4" s="26"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="32" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B5" s="32"/>
       <c r="C5" s="32"/>
@@ -8012,25 +8007,25 @@
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" s="34" t="s">
         <v>123</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="C7" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="D7" s="33" t="s">
         <v>125</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>126</v>
       </c>
       <c r="E7" s="33" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="33" t="s">
+        <v>126</v>
+      </c>
+      <c r="G7" s="33" t="s">
         <v>127</v>
-      </c>
-      <c r="G7" s="33" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
@@ -8038,16 +8033,16 @@
         <v>1.0</v>
       </c>
       <c r="B8" s="36" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" s="36" t="s">
         <v>129</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="D8" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="D8" s="37" t="s">
+      <c r="E8" s="38" t="s">
         <v>131</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>132</v>
       </c>
       <c r="F8" s="39"/>
       <c r="G8" s="40"/>
@@ -8057,16 +8052,16 @@
         <v>2.0</v>
       </c>
       <c r="B9" s="42" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C9" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D9" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="E9" s="44" t="s">
         <v>133</v>
-      </c>
-      <c r="D9" s="43" t="s">
-        <v>131</v>
-      </c>
-      <c r="E9" s="44" t="s">
-        <v>134</v>
       </c>
       <c r="F9" s="45"/>
       <c r="G9" s="40"/>
@@ -8076,16 +8071,16 @@
         <v>3.0</v>
       </c>
       <c r="B10" s="47" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" s="47" t="s">
         <v>135</v>
       </c>
-      <c r="C10" s="47" t="s">
+      <c r="D10" s="48" t="s">
         <v>136</v>
       </c>
-      <c r="D10" s="48" t="s">
+      <c r="E10" s="49" t="s">
         <v>137</v>
-      </c>
-      <c r="E10" s="49" t="s">
-        <v>138</v>
       </c>
       <c r="F10" s="50"/>
       <c r="G10" s="51"/>
@@ -8095,10 +8090,10 @@
       <c r="B11" s="36"/>
       <c r="C11" s="36"/>
       <c r="D11" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="E11" s="38" t="s">
         <v>139</v>
-      </c>
-      <c r="E11" s="38" t="s">
-        <v>140</v>
       </c>
       <c r="F11" s="52"/>
       <c r="G11" s="53"/>
@@ -8108,16 +8103,16 @@
         <v>4.0</v>
       </c>
       <c r="B12" s="55" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="C12" s="55" t="s">
+      <c r="D12" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="D12" s="56" t="s">
+      <c r="E12" s="57" t="s">
         <v>143</v>
-      </c>
-      <c r="E12" s="57" t="s">
-        <v>144</v>
       </c>
       <c r="F12" s="58"/>
       <c r="G12" s="59"/>
@@ -8127,10 +8122,10 @@
       <c r="B13" s="36"/>
       <c r="C13" s="36"/>
       <c r="D13" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="E13" s="38" t="s">
         <v>145</v>
-      </c>
-      <c r="E13" s="38" t="s">
-        <v>146</v>
       </c>
       <c r="F13" s="39"/>
       <c r="G13" s="53"/>
@@ -8140,16 +8135,16 @@
         <v>5.0</v>
       </c>
       <c r="B14" s="55" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C14" s="55" t="s">
+        <v>146</v>
+      </c>
+      <c r="D14" s="56" t="s">
         <v>147</v>
       </c>
-      <c r="D14" s="56" t="s">
+      <c r="E14" s="57" t="s">
         <v>148</v>
-      </c>
-      <c r="E14" s="57" t="s">
-        <v>149</v>
       </c>
       <c r="F14" s="58"/>
       <c r="G14" s="59"/>
@@ -8159,13 +8154,13 @@
       <c r="B15" s="36"/>
       <c r="C15" s="36"/>
       <c r="D15" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E15" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="F15" s="60" t="s">
         <v>150</v>
-      </c>
-      <c r="F15" s="60" t="s">
-        <v>151</v>
       </c>
       <c r="G15" s="53"/>
     </row>
@@ -8174,16 +8169,16 @@
         <v>6.0</v>
       </c>
       <c r="B16" s="55" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="C16" s="55" t="s">
-        <v>142</v>
-      </c>
       <c r="D16" s="56" t="s">
+        <v>151</v>
+      </c>
+      <c r="E16" s="57" t="s">
         <v>152</v>
-      </c>
-      <c r="E16" s="57" t="s">
-        <v>153</v>
       </c>
       <c r="F16" s="61"/>
       <c r="G16" s="59"/>
@@ -8193,10 +8188,10 @@
       <c r="B17" s="36"/>
       <c r="C17" s="36"/>
       <c r="D17" s="37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F17" s="62"/>
       <c r="G17" s="53"/>

</xml_diff>